<commit_message>
upload Khách Hàng, xử  lí Upsert cho các chức năng upload
</commit_message>
<xml_diff>
--- a/API/Resources/Template/KhachHang/Report.xlsx
+++ b/API/Resources/Template/KhachHang/Report.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Lỗi</t>
   </si>
@@ -49,6 +49,12 @@
   </si>
   <si>
     <t>&amp;=result.Email</t>
+  </si>
+  <si>
+    <t>Mã Khách Hàng</t>
+  </si>
+  <si>
+    <t>&amp;=result.Ma_KH</t>
   </si>
 </sst>
 </file>
@@ -113,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -135,6 +141,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,47 +429,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="8"/>
+    <col min="1" max="2" width="20.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="22" style="3" customWidth="1"/>
+    <col min="6" max="6" width="35.5703125" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
bỏ trường Ten_SP và Dvt trong bảng ChiTietDonHang, chỉnh sửa các hàm liên quan
</commit_message>
<xml_diff>
--- a/API/Resources/Template/KhachHang/Report.xlsx
+++ b/API/Resources/Template/KhachHang/Report.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D661E18-8C30-4198-85D8-40AB6C5B5F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -142,7 +143,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,13 +429,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" style="2" customWidth="1"/>
     <col min="5" max="5" width="22" style="3" customWidth="1"/>
     <col min="6" max="6" width="35.5703125" style="8" customWidth="1"/>
   </cols>
@@ -447,10 +448,10 @@
         <v>3</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>5</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>6</v>
@@ -466,11 +467,11 @@
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>9</v>

</xml_diff>